<commit_message>
feat: add shopping list API
</commit_message>
<xml_diff>
--- a/doc/02_DB設計書.xlsx
+++ b/doc/02_DB設計書.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\junya\Desktop\My_Dev\MenuMate\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\junya\Desktop\My_Dev\MenuMate\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B31B5372-0C7F-4096-9935-0319DA1B8BF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13811515-DBA7-4DD8-9D4F-AF2AC7FE091B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43170" yWindow="3735" windowWidth="23040" windowHeight="12120" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DB一覧" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="107">
   <si>
     <t>テーブル名</t>
     <rPh sb="4" eb="5">
@@ -358,6 +358,10 @@
   </si>
   <si>
     <t>お気に入り</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   "mealPlanId":"20260930-dinner"</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
@@ -501,7 +505,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -514,8 +518,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -1131,11 +1133,6 @@
         <v>71</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
-      <c r="A17" s="13"/>
-      <c r="B17" s="13"/>
-      <c r="C17" s="13"/>
-    </row>
     <row r="20" spans="1:3">
       <c r="A20" s="3" t="s">
         <v>72</v>
@@ -1589,11 +1586,6 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
-      <c r="B2" t="s">
-        <v>54</v>
-      </c>
-    </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
         <v>12</v>
@@ -1629,84 +1621,80 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
-        <v>55</v>
+        <v>96</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>8</v>
+        <v>24</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
-        <v>96</v>
+        <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C8" s="1" t="s">
         <v>70</v>
       </c>
     </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" s="4"/>
+      <c r="C10" s="5"/>
+    </row>
     <row r="11" spans="1:3">
-      <c r="A11" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B11" s="4"/>
-      <c r="C11" s="5"/>
+      <c r="A11" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B11" s="7"/>
+      <c r="C11" s="8"/>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B12" s="12"/>
+        <v>106</v>
+      </c>
+      <c r="B12" s="7"/>
       <c r="C12" s="8"/>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="B13" s="12"/>
+      <c r="B13" s="7"/>
       <c r="C13" s="8"/>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="B14" s="12"/>
+      <c r="B14" s="7"/>
       <c r="C14" s="8"/>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B15" s="12"/>
+      <c r="B15" s="7"/>
       <c r="C15" s="8"/>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B16" s="12"/>
+      <c r="B16" s="7"/>
       <c r="C16" s="8"/>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="B17" s="12"/>
+      <c r="B17" s="7"/>
       <c r="C17" s="8"/>
     </row>
     <row r="18" spans="1:3">
@@ -1719,5 +1707,6 @@
   </sheetData>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>